<commit_message>
Rename Development-category milestone Build Completed to Development Completed
Matches the updated Milestone_Lookup_Table.xlsx source data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Milestone_Lookup_Table.xlsx
+++ b/Milestone_Lookup_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peer/Documents/Claude/Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956333D3-5D31-B741-A699-13905C15E1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE0FFC1-6780-B549-A509-6998D0E12A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,9 +40,6 @@
     <t>Design Defined</t>
   </si>
   <si>
-    <t>Build Completed</t>
-  </si>
-  <si>
     <t>Ready for SIT</t>
   </si>
   <si>
@@ -89,6 +86,9 @@
   </si>
   <si>
     <t>Activity Completed</t>
+  </si>
+  <si>
+    <t>Development Completed</t>
   </si>
 </sst>
 </file>
@@ -107,10 +107,12 @@
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -483,7 +485,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -491,7 +493,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -499,7 +501,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -507,52 +509,52 @@
         <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>5</v>
@@ -560,74 +562,74 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync DEFAULT_CATEGORIES' Artefact template against the updated lookup table
Milestone_Lookup_Table.xlsx gained a new 4th Artefact milestone, "Artefact
Published / Distributed" (after Draft Completed / Ready for Review /
Artefact Approved). Only affects what a brand-new install seeds; existing
programmes' own Artefact categories are untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Milestone_Lookup_Table.xlsx
+++ b/Milestone_Lookup_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peer/Documents/Claude/Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F903B112-251B-964C-8D1A-AC8CC5AFF872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44373BCD-43EA-6A42-81F2-CA6F44AFF4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="23">
   <si>
     <t>Type</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>Development Completed</t>
+  </si>
+  <si>
+    <t>Artefact Published / Distributed</t>
   </si>
 </sst>
 </file>
@@ -438,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -535,10 +538,10 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -546,7 +549,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -554,7 +557,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -562,7 +565,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -570,7 +573,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -578,15 +581,15 @@
         <v>13</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -594,7 +597,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -602,7 +605,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -610,7 +613,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -618,6 +621,14 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync DEFAULT_CATEGORIES with the updated milestone lookup table
Activity's first milestone renamed from "Activity Defined" to "Activity
Planned" in Milestone_Lookup_Table.xlsx. Development, Artefact, and
Integration are unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Milestone_Lookup_Table.xlsx
+++ b/Milestone_Lookup_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peer/Documents/Claude/Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF9A9F4-0117-074F-9456-73F525A78007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45E26E5-F6C7-264F-ABC8-30F51AD07B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,9 +70,6 @@
     <t>Activity</t>
   </si>
   <si>
-    <t>Activity Defined</t>
-  </si>
-  <si>
     <t>Activity Prepared</t>
   </si>
   <si>
@@ -89,6 +86,9 @@
   </si>
   <si>
     <t>Artefact Published</t>
+  </si>
+  <si>
+    <t>Activity Planned</t>
   </si>
 </sst>
 </file>
@@ -485,7 +485,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -541,7 +541,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -565,7 +565,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -597,7 +597,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -605,7 +605,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -613,7 +613,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -621,7 +621,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -629,7 +629,7 @@
         <v>15</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update default category milestones from the refreshed lookup table
Milestone_Lookup_Table.xlsx replaced Development's "Ready for SIT"/"Ready
for E2E" pair with a single "Ready for Testing" step, dropped the
Integration category, and added a new Dependency category — reflected here
in DEFAULT_CATEGORIES, which only seeds a fresh programme's out-of-the-box
categories.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Milestone_Lookup_Table.xlsx
+++ b/Milestone_Lookup_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peer/Documents/Claude/Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45E26E5-F6C7-264F-ABC8-30F51AD07B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CB44E1-C7AB-6748-88A2-6CD915F504BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="23">
   <si>
     <t>Type</t>
   </si>
@@ -40,12 +40,6 @@
     <t>Design Defined</t>
   </si>
   <si>
-    <t>Ready for SIT</t>
-  </si>
-  <si>
-    <t>Ready for E2E</t>
-  </si>
-  <si>
     <t>Deployment Completed</t>
   </si>
   <si>
@@ -61,12 +55,6 @@
     <t>Artefact Approved</t>
   </si>
   <si>
-    <t>Integration</t>
-  </si>
-  <si>
-    <t>Interface Specification Agreed</t>
-  </si>
-  <si>
     <t>Activity</t>
   </si>
   <si>
@@ -89,6 +77,18 @@
   </si>
   <si>
     <t>Activity Planned</t>
+  </si>
+  <si>
+    <t>Ready for Testing</t>
+  </si>
+  <si>
+    <t>Delivery Commitment Confirmed</t>
+  </si>
+  <si>
+    <t>Dependency Delivered</t>
+  </si>
+  <si>
+    <t>Dependency</t>
   </si>
 </sst>
 </file>
@@ -441,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -485,7 +485,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -493,7 +493,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -501,12 +501,12 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
@@ -514,122 +514,106 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>